<commit_message>
Actualizar monitoreo SISE emergencias
</commit_message>
<xml_diff>
--- a/emergencias/assets/reportes/Reporte_sectorial_MIDESO.xlsx
+++ b/emergencias/assets/reportes/Reporte_sectorial_MIDESO.xlsx
@@ -1411,7 +1411,7 @@
       <c r="C5" s="6" t="n"/>
       <c r="D5" s="69" t="inlineStr">
         <is>
-          <t>15-07-2026, 17hrs</t>
+          <t>15-07-2026, 16:58 hrs</t>
         </is>
       </c>
       <c r="E5" s="70" t="n"/>
@@ -1571,11 +1571,11 @@
         </is>
       </c>
       <c r="E14" s="36" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="F14" s="73" t="n"/>
       <c r="G14" s="36" t="n">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="H14" s="73" t="n"/>
       <c r="I14" s="6" t="n"/>
@@ -1591,11 +1591,11 @@
         </is>
       </c>
       <c r="E15" s="36" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="F15" s="73" t="n"/>
       <c r="G15" s="36" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H15" s="73" t="n"/>
       <c r="I15" s="6" t="n"/>
@@ -1611,11 +1611,11 @@
         </is>
       </c>
       <c r="E16" s="36" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="F16" s="73" t="n"/>
       <c r="G16" s="36" t="n">
-        <v>161</v>
+        <v>0</v>
       </c>
       <c r="H16" s="73" t="n"/>
       <c r="I16" s="6" t="n"/>
@@ -1631,11 +1631,11 @@
         </is>
       </c>
       <c r="E17" s="36" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="F17" s="73" t="n"/>
       <c r="G17" s="36" t="n">
-        <v>103</v>
+        <v>0</v>
       </c>
       <c r="H17" s="73" t="n"/>
       <c r="I17" s="6" t="n"/>
@@ -1651,11 +1651,11 @@
         </is>
       </c>
       <c r="E18" s="36" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="F18" s="73" t="n"/>
       <c r="G18" s="36" t="n">
-        <v>139</v>
+        <v>0</v>
       </c>
       <c r="H18" s="73" t="n"/>
       <c r="I18" s="6" t="n"/>
@@ -1671,11 +1671,11 @@
         </is>
       </c>
       <c r="E19" s="36" t="n">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="F19" s="73" t="n"/>
       <c r="G19" s="36" t="n">
-        <v>214</v>
+        <v>0</v>
       </c>
       <c r="H19" s="73" t="n"/>
       <c r="I19" s="6" t="n"/>
@@ -1691,11 +1691,11 @@
         </is>
       </c>
       <c r="E20" s="36" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="F20" s="73" t="n"/>
       <c r="G20" s="36" t="n">
-        <v>173</v>
+        <v>0</v>
       </c>
       <c r="H20" s="73" t="n"/>
       <c r="I20" s="6" t="n"/>
@@ -1711,11 +1711,11 @@
         </is>
       </c>
       <c r="E21" s="36" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="F21" s="73" t="n"/>
       <c r="G21" s="36" t="n">
-        <v>186</v>
+        <v>0</v>
       </c>
       <c r="H21" s="73" t="n"/>
       <c r="I21" s="6" t="n"/>
@@ -1731,11 +1731,11 @@
         </is>
       </c>
       <c r="E22" s="36" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="F22" s="73" t="n"/>
       <c r="G22" s="36" t="n">
-        <v>122</v>
+        <v>0</v>
       </c>
       <c r="H22" s="73" t="n"/>
       <c r="I22" s="6" t="n"/>
@@ -1751,11 +1751,11 @@
         </is>
       </c>
       <c r="E23" s="36" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="F23" s="73" t="n"/>
       <c r="G23" s="36" t="n">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="H23" s="73" t="n"/>
       <c r="I23" s="6" t="n"/>
@@ -1771,11 +1771,11 @@
         </is>
       </c>
       <c r="E24" s="36" t="n">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="F24" s="73" t="n"/>
       <c r="G24" s="36" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="H24" s="73" t="n"/>
       <c r="I24" s="6" t="n"/>

</xml_diff>